<commit_message>
feat(planes): actualizacion global modular de todos los planes de vuelo de clientes
</commit_message>
<xml_diff>
--- a/planes/rocio/Plantillas/08_Cancionero_Inventario_y_Plan_Clases_Voz_Caleidoscopio.xlsx
+++ b/planes/rocio/Plantillas/08_Cancionero_Inventario_y_Plan_Clases_Voz_Caleidoscopio.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancionero e Inventario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora y Composición" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estructura 70min &amp; Bitácora" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Certificación Feldenkrais" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -868,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -884,32 +884,57 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Lugar (Playa / Sala)</t>
+          <t>Lugar (Playa/Sala)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Fase 1: Somática Feldenkrais</t>
+          <t>Fase 1 (20m): Vocalizar sin notas</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Fase 2: Roy Hart / Técnica</t>
+          <t>Pausa (2m)</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Fase 3: Canción Trabajada</t>
+          <t>Fase 2 (10m): Apertura Corporal</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Fase 4: Idea Composición / Tarea</t>
+          <t>Pausa (2m)</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
         <is>
-          <t>Audio Recibido</t>
+          <t>Fase 3 (15m): Lectura 8 Compases</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Pausa (2m)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Fase 4 (5m): Escucha &amp; Análisis</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Pausa (2m)</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Fase 5 (10m): Apertura &amp; Cierre</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Audio Tarea Recibido</t>
         </is>
       </c>
     </row>

</xml_diff>